<commit_message>
Update ETL pipeline, chatbot, ML models, and Streamlit app
</commit_message>
<xml_diff>
--- a/dataset/synthesize/assignment_submissions_progress_synthetic_numpy.xlsx
+++ b/dataset/synthesize/assignment_submissions_progress_synthetic_numpy.xlsx
@@ -474,7 +474,7 @@
     <col width="35" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
-    <col width="35" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
     <col width="24" customWidth="1" min="7" max="7"/>
     <col width="24" customWidth="1" min="8" max="8"/>
@@ -569,7 +569,7 @@
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>Meetraj Solanki, Keval Sanghani, Aditya Patel, Mukesh Goswami, Chandan Kamal, Ganpat Prajapati, Deepak Khatri, Shrey Savaliya, Vidhan Padsala, Keyur Chaniyara, Yatree Ladani</t>
+          <t>Chandan Kamal</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
@@ -631,7 +631,7 @@
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t>Meetraj Solanki, Keval Sanghani, Aditya Patel, Mukesh Goswami, Chandan Kamal, Ganpat Prajapati, Deepak Khatri, Shrey Savaliya, Vidhan Padsala, Keyur Chaniyara, Yatree Ladani</t>
+          <t>Vidhan Padsala</t>
         </is>
       </c>
       <c r="F3" s="5" t="inlineStr">
@@ -693,7 +693,7 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>Meetraj Solanki, Keval Sanghani, Aditya Patel, Mukesh Goswami, Chandan Kamal, Ganpat Prajapati, Deepak Khatri, Shrey Savaliya, Vidhan Padsala, Keyur Chaniyara, Yatree Ladani</t>
+          <t>Deepak Khatri</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
@@ -755,7 +755,7 @@
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>Meetraj Solanki, Keval Sanghani, Aditya Patel, Mukesh Goswami, Chandan Kamal, Ganpat Prajapati, Deepak Khatri, Shrey Savaliya, Vidhan Padsala, Keyur Chaniyara, Yatree Ladani</t>
+          <t>Chandan Kamal</t>
         </is>
       </c>
       <c r="F5" s="5" t="inlineStr">
@@ -817,7 +817,7 @@
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>Meetraj Solanki, Keval Sanghani, Aditya Patel, Mukesh Goswami, Chandan Kamal, Ganpat Prajapati, Deepak Khatri, Shrey Savaliya, Vidhan Padsala, Keyur Chaniyara, Yatree Ladani</t>
+          <t>Aditya Patel</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
@@ -879,7 +879,7 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>Meetraj Solanki, Keval Sanghani, Aditya Patel, Mukesh Goswami, Chandan Kamal, Ganpat Prajapati, Deepak Khatri, Shrey Savaliya, Vidhan Padsala, Keyur Chaniyara, Yatree Ladani</t>
+          <t>Mukesh Goswami</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
@@ -941,7 +941,7 @@
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>Meetraj Solanki, Keval Sanghani, Aditya Patel, Mukesh Goswami, Chandan Kamal, Ganpat Prajapati, Deepak Khatri, Shrey Savaliya, Vidhan Padsala, Keyur Chaniyara, Yatree Ladani</t>
+          <t>Yatree Ladani</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
@@ -1003,7 +1003,7 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>Meetraj Solanki, Keval Sanghani, Aditya Patel, Mukesh Goswami, Chandan Kamal, Ganpat Prajapati, Deepak Khatri, Shrey Savaliya, Vidhan Padsala, Keyur Chaniyara, Yatree Ladani</t>
+          <t>Keval Sanghani</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
@@ -1065,7 +1065,7 @@
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>Meetraj Solanki, Keval Sanghani, Aditya Patel, Mukesh Goswami, Chandan Kamal, Ganpat Prajapati, Deepak Khatri, Shrey Savaliya, Vidhan Padsala, Keyur Chaniyara, Yatree Ladani</t>
+          <t>Deepak Khatri</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
@@ -1127,7 +1127,7 @@
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>Meetraj Solanki, Keval Sanghani, Aditya Patel, Mukesh Goswami, Chandan Kamal, Ganpat Prajapati, Deepak Khatri, Shrey Savaliya, Vidhan Padsala, Keyur Chaniyara, Yatree Ladani</t>
+          <t>Keval Sanghani</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
@@ -1189,7 +1189,7 @@
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>Meetraj Solanki, Keval Sanghani, Aditya Patel, Mukesh Goswami, Chandan Kamal, Ganpat Prajapati, Deepak Khatri, Shrey Savaliya, Vidhan Padsala, Keyur Chaniyara, Yatree Ladani</t>
+          <t>Ganpat Prajapati</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
@@ -1251,7 +1251,7 @@
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>Meetraj Solanki, Keval Sanghani, Aditya Patel, Mukesh Goswami, Chandan Kamal, Ganpat Prajapati, Deepak Khatri, Shrey Savaliya, Vidhan Padsala, Keyur Chaniyara, Yatree Ladani</t>
+          <t>Meetraj Solanki</t>
         </is>
       </c>
       <c r="F13" s="5" t="inlineStr">
@@ -1313,7 +1313,7 @@
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>Meetraj Solanki, Keval Sanghani, Aditya Patel, Mukesh Goswami, Chandan Kamal, Ganpat Prajapati, Deepak Khatri, Shrey Savaliya, Vidhan Padsala, Keyur Chaniyara, Yatree Ladani</t>
+          <t>Shrey Savaliya</t>
         </is>
       </c>
       <c r="F14" s="3" t="inlineStr">
@@ -1375,7 +1375,7 @@
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>Meetraj Solanki, Keval Sanghani, Aditya Patel, Mukesh Goswami, Chandan Kamal, Ganpat Prajapati, Deepak Khatri, Shrey Savaliya, Vidhan Padsala, Keyur Chaniyara, Yatree Ladani</t>
+          <t>Deepak Khatri</t>
         </is>
       </c>
       <c r="F15" s="5" t="inlineStr">
@@ -1437,7 +1437,7 @@
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>Meetraj Solanki, Keval Sanghani, Aditya Patel, Mukesh Goswami, Chandan Kamal, Ganpat Prajapati, Deepak Khatri, Shrey Savaliya, Vidhan Padsala, Keyur Chaniyara, Yatree Ladani</t>
+          <t>Keyur Chaniyara</t>
         </is>
       </c>
       <c r="F16" s="3" t="inlineStr">
@@ -1499,7 +1499,7 @@
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>Meetraj Solanki, Keval Sanghani, Aditya Patel, Mukesh Goswami, Chandan Kamal, Ganpat Prajapati, Deepak Khatri, Shrey Savaliya, Vidhan Padsala, Keyur Chaniyara, Yatree Ladani</t>
+          <t>Mukesh Goswami</t>
         </is>
       </c>
       <c r="F17" s="5" t="inlineStr">
@@ -1561,7 +1561,7 @@
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>Meetraj Solanki, Keval Sanghani, Aditya Patel, Mukesh Goswami, Chandan Kamal, Ganpat Prajapati, Deepak Khatri, Shrey Savaliya, Vidhan Padsala, Keyur Chaniyara, Yatree Ladani</t>
+          <t>Chandan Kamal</t>
         </is>
       </c>
       <c r="F18" s="3" t="inlineStr">
@@ -1623,7 +1623,7 @@
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t>Meetraj Solanki, Keval Sanghani, Aditya Patel, Mukesh Goswami, Chandan Kamal, Ganpat Prajapati, Deepak Khatri, Shrey Savaliya, Vidhan Padsala, Keyur Chaniyara, Yatree Ladani</t>
+          <t>Yatree Ladani</t>
         </is>
       </c>
       <c r="F19" s="5" t="inlineStr">
@@ -1685,7 +1685,7 @@
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>Meetraj Solanki, Keval Sanghani, Aditya Patel, Mukesh Goswami, Chandan Kamal, Ganpat Prajapati, Deepak Khatri, Shrey Savaliya, Vidhan Padsala, Keyur Chaniyara, Yatree Ladani</t>
+          <t>Vidhan Padsala</t>
         </is>
       </c>
       <c r="F20" s="3" t="inlineStr">
@@ -1747,7 +1747,7 @@
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t>Meetraj Solanki, Keval Sanghani, Aditya Patel, Mukesh Goswami, Chandan Kamal, Ganpat Prajapati, Deepak Khatri, Shrey Savaliya, Vidhan Padsala, Keyur Chaniyara, Yatree Ladani</t>
+          <t>Meetraj Solanki</t>
         </is>
       </c>
       <c r="F21" s="5" t="inlineStr">
@@ -1809,7 +1809,7 @@
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>Meetraj Solanki, Keval Sanghani, Aditya Patel, Mukesh Goswami, Chandan Kamal, Ganpat Prajapati, Deepak Khatri, Shrey Savaliya, Vidhan Padsala, Keyur Chaniyara, Yatree Ladani</t>
+          <t>Aditya Patel</t>
         </is>
       </c>
       <c r="F22" s="3" t="inlineStr">
@@ -1871,7 +1871,7 @@
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t>Meetraj Solanki, Keval Sanghani, Aditya Patel, Mukesh Goswami, Chandan Kamal, Ganpat Prajapati, Deepak Khatri, Shrey Savaliya, Vidhan Padsala, Keyur Chaniyara, Yatree Ladani</t>
+          <t>Mukesh Goswami</t>
         </is>
       </c>
       <c r="F23" s="5" t="inlineStr">
@@ -1933,7 +1933,7 @@
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>Meetraj Solanki, Keval Sanghani, Aditya Patel, Mukesh Goswami, Chandan Kamal, Ganpat Prajapati, Deepak Khatri, Shrey Savaliya, Vidhan Padsala, Keyur Chaniyara, Yatree Ladani</t>
+          <t>Yatree Ladani</t>
         </is>
       </c>
       <c r="F24" s="3" t="inlineStr">
@@ -1995,7 +1995,7 @@
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t>Meetraj Solanki, Keval Sanghani, Aditya Patel, Mukesh Goswami, Chandan Kamal, Ganpat Prajapati, Deepak Khatri, Shrey Savaliya, Vidhan Padsala, Keyur Chaniyara, Yatree Ladani</t>
+          <t>Deepak Khatri</t>
         </is>
       </c>
       <c r="F25" s="5" t="inlineStr">
@@ -2057,7 +2057,7 @@
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>Meetraj Solanki, Keval Sanghani, Aditya Patel, Mukesh Goswami, Chandan Kamal, Ganpat Prajapati, Deepak Khatri, Shrey Savaliya, Vidhan Padsala, Keyur Chaniyara, Yatree Ladani</t>
+          <t>Keval Sanghani</t>
         </is>
       </c>
       <c r="F26" s="3" t="inlineStr">
@@ -2119,7 +2119,7 @@
       </c>
       <c r="E27" s="5" t="inlineStr">
         <is>
-          <t>Meetraj Solanki, Keval Sanghani, Aditya Patel, Mukesh Goswami, Chandan Kamal, Ganpat Prajapati, Deepak Khatri, Shrey Savaliya, Vidhan Padsala, Keyur Chaniyara, Yatree Ladani</t>
+          <t>Ganpat Prajapati</t>
         </is>
       </c>
       <c r="F27" s="5" t="inlineStr">
@@ -2181,7 +2181,7 @@
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>Meetraj Solanki, Keval Sanghani, Aditya Patel, Mukesh Goswami, Chandan Kamal, Ganpat Prajapati, Deepak Khatri, Shrey Savaliya, Vidhan Padsala, Keyur Chaniyara, Yatree Ladani</t>
+          <t>Meetraj Solanki</t>
         </is>
       </c>
       <c r="F28" s="3" t="inlineStr">
@@ -2243,7 +2243,7 @@
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t>Meetraj Solanki, Keval Sanghani, Aditya Patel, Mukesh Goswami, Chandan Kamal, Ganpat Prajapati, Deepak Khatri, Shrey Savaliya, Vidhan Padsala, Keyur Chaniyara, Yatree Ladani</t>
+          <t>Shrey Savaliya</t>
         </is>
       </c>
       <c r="F29" s="5" t="inlineStr">
@@ -2305,7 +2305,7 @@
       </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t>Meetraj Solanki, Keval Sanghani, Aditya Patel, Mukesh Goswami, Chandan Kamal, Ganpat Prajapati, Deepak Khatri, Shrey Savaliya, Vidhan Padsala, Keyur Chaniyara, Yatree Ladani</t>
+          <t>Keyur Chaniyara</t>
         </is>
       </c>
       <c r="F30" s="3" t="inlineStr">
@@ -2367,7 +2367,7 @@
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t>Meetraj Solanki, Keval Sanghani, Aditya Patel, Mukesh Goswami, Chandan Kamal, Ganpat Prajapati, Deepak Khatri, Shrey Savaliya, Vidhan Padsala, Keyur Chaniyara, Yatree Ladani</t>
+          <t>Chandan Kamal</t>
         </is>
       </c>
       <c r="F31" s="5" t="inlineStr">
@@ -2429,7 +2429,7 @@
       </c>
       <c r="E32" s="3" t="inlineStr">
         <is>
-          <t>Meetraj Solanki, Keval Sanghani, Aditya Patel, Mukesh Goswami, Chandan Kamal, Ganpat Prajapati, Deepak Khatri, Shrey Savaliya, Vidhan Padsala, Keyur Chaniyara, Yatree Ladani</t>
+          <t>Vidhan Padsala</t>
         </is>
       </c>
       <c r="F32" s="3" t="inlineStr">
@@ -2491,7 +2491,7 @@
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t>Meetraj Solanki, Keval Sanghani, Aditya Patel, Mukesh Goswami, Chandan Kamal, Ganpat Prajapati, Deepak Khatri, Shrey Savaliya, Vidhan Padsala, Keyur Chaniyara, Yatree Ladani</t>
+          <t>Aditya Patel</t>
         </is>
       </c>
       <c r="F33" s="5" t="inlineStr">
@@ -2553,7 +2553,7 @@
       </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
-          <t>Meetraj Solanki, Keval Sanghani, Aditya Patel, Mukesh Goswami, Chandan Kamal, Ganpat Prajapati, Deepak Khatri, Shrey Savaliya, Vidhan Padsala, Keyur Chaniyara, Yatree Ladani</t>
+          <t>Vidhan Padsala</t>
         </is>
       </c>
       <c r="F34" s="3" t="inlineStr">
@@ -2615,7 +2615,7 @@
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t>Meetraj Solanki, Keval Sanghani, Aditya Patel, Mukesh Goswami, Chandan Kamal, Ganpat Prajapati, Deepak Khatri, Shrey Savaliya, Vidhan Padsala, Keyur Chaniyara, Yatree Ladani</t>
+          <t>Keyur Chaniyara</t>
         </is>
       </c>
       <c r="F35" s="5" t="inlineStr">
@@ -2677,7 +2677,7 @@
       </c>
       <c r="E36" s="3" t="inlineStr">
         <is>
-          <t>Meetraj Solanki, Keval Sanghani, Aditya Patel, Mukesh Goswami, Chandan Kamal, Ganpat Prajapati, Deepak Khatri, Shrey Savaliya, Vidhan Padsala, Keyur Chaniyara, Yatree Ladani</t>
+          <t>Ganpat Prajapati</t>
         </is>
       </c>
       <c r="F36" s="3" t="inlineStr">
@@ -2739,7 +2739,7 @@
       </c>
       <c r="E37" s="5" t="inlineStr">
         <is>
-          <t>Meetraj Solanki, Keval Sanghani, Aditya Patel, Mukesh Goswami, Chandan Kamal, Ganpat Prajapati, Deepak Khatri, Shrey Savaliya, Vidhan Padsala, Keyur Chaniyara, Yatree Ladani</t>
+          <t>Deepak Khatri</t>
         </is>
       </c>
       <c r="F37" s="5" t="inlineStr">
@@ -2801,7 +2801,7 @@
       </c>
       <c r="E38" s="3" t="inlineStr">
         <is>
-          <t>Meetraj Solanki, Keval Sanghani, Aditya Patel, Mukesh Goswami, Chandan Kamal, Ganpat Prajapati, Deepak Khatri, Shrey Savaliya, Vidhan Padsala, Keyur Chaniyara, Yatree Ladani</t>
+          <t>Mukesh Goswami</t>
         </is>
       </c>
       <c r="F38" s="3" t="inlineStr">
@@ -2863,7 +2863,7 @@
       </c>
       <c r="E39" s="5" t="inlineStr">
         <is>
-          <t>Meetraj Solanki, Keval Sanghani, Aditya Patel, Mukesh Goswami, Chandan Kamal, Ganpat Prajapati, Deepak Khatri, Shrey Savaliya, Vidhan Padsala, Keyur Chaniyara, Yatree Ladani</t>
+          <t>Yatree Ladani</t>
         </is>
       </c>
       <c r="F39" s="5" t="inlineStr">
@@ -2925,7 +2925,7 @@
       </c>
       <c r="E40" s="3" t="inlineStr">
         <is>
-          <t>Meetraj Solanki, Keval Sanghani, Aditya Patel, Mukesh Goswami, Chandan Kamal, Ganpat Prajapati, Deepak Khatri, Shrey Savaliya, Vidhan Padsala, Keyur Chaniyara, Yatree Ladani</t>
+          <t>Deepak Khatri</t>
         </is>
       </c>
       <c r="F40" s="3" t="inlineStr">
@@ -2987,7 +2987,7 @@
       </c>
       <c r="E41" s="5" t="inlineStr">
         <is>
-          <t>Meetraj Solanki, Keval Sanghani, Aditya Patel, Mukesh Goswami, Chandan Kamal, Ganpat Prajapati, Deepak Khatri, Shrey Savaliya, Vidhan Padsala, Keyur Chaniyara, Yatree Ladani</t>
+          <t>Yatree Ladani</t>
         </is>
       </c>
       <c r="F41" s="5" t="inlineStr">
@@ -3049,7 +3049,7 @@
       </c>
       <c r="E42" s="3" t="inlineStr">
         <is>
-          <t>Meetraj Solanki, Keval Sanghani, Aditya Patel, Mukesh Goswami, Chandan Kamal, Ganpat Prajapati, Deepak Khatri, Shrey Savaliya, Vidhan Padsala, Keyur Chaniyara, Yatree Ladani</t>
+          <t>Keval Sanghani</t>
         </is>
       </c>
       <c r="F42" s="3" t="inlineStr">
@@ -3111,7 +3111,7 @@
       </c>
       <c r="E43" s="5" t="inlineStr">
         <is>
-          <t>Meetraj Solanki, Keval Sanghani, Aditya Patel, Mukesh Goswami, Chandan Kamal, Ganpat Prajapati, Deepak Khatri, Shrey Savaliya, Vidhan Padsala, Keyur Chaniyara, Yatree Ladani</t>
+          <t>Meetraj Solanki</t>
         </is>
       </c>
       <c r="F43" s="5" t="inlineStr">
@@ -3173,7 +3173,7 @@
       </c>
       <c r="E44" s="3" t="inlineStr">
         <is>
-          <t>Meetraj Solanki, Keval Sanghani, Aditya Patel, Mukesh Goswami, Chandan Kamal, Ganpat Prajapati, Deepak Khatri, Shrey Savaliya, Vidhan Padsala, Keyur Chaniyara, Yatree Ladani</t>
+          <t>Aditya Patel</t>
         </is>
       </c>
       <c r="F44" s="3" t="inlineStr">
@@ -3235,7 +3235,7 @@
       </c>
       <c r="E45" s="5" t="inlineStr">
         <is>
-          <t>Meetraj Solanki, Keval Sanghani, Aditya Patel, Mukesh Goswami, Chandan Kamal, Ganpat Prajapati, Deepak Khatri, Shrey Savaliya, Vidhan Padsala, Keyur Chaniyara, Yatree Ladani</t>
+          <t>Vidhan Padsala</t>
         </is>
       </c>
       <c r="F45" s="5" t="inlineStr">
@@ -3297,7 +3297,7 @@
       </c>
       <c r="E46" s="3" t="inlineStr">
         <is>
-          <t>Meetraj Solanki, Keval Sanghani, Aditya Patel, Mukesh Goswami, Chandan Kamal, Ganpat Prajapati, Deepak Khatri, Shrey Savaliya, Vidhan Padsala, Keyur Chaniyara, Yatree Ladani</t>
+          <t>Keyur Chaniyara</t>
         </is>
       </c>
       <c r="F46" s="3" t="inlineStr">
@@ -3359,7 +3359,7 @@
       </c>
       <c r="E47" s="5" t="inlineStr">
         <is>
-          <t>Meetraj Solanki, Keval Sanghani, Aditya Patel, Mukesh Goswami, Chandan Kamal, Ganpat Prajapati, Deepak Khatri, Shrey Savaliya, Vidhan Padsala, Keyur Chaniyara, Yatree Ladani</t>
+          <t>Ganpat Prajapati</t>
         </is>
       </c>
       <c r="F47" s="5" t="inlineStr">
@@ -3421,7 +3421,7 @@
       </c>
       <c r="E48" s="3" t="inlineStr">
         <is>
-          <t>Meetraj Solanki, Keval Sanghani, Aditya Patel, Mukesh Goswami, Chandan Kamal, Ganpat Prajapati, Deepak Khatri, Shrey Savaliya, Vidhan Padsala, Keyur Chaniyara, Yatree Ladani</t>
+          <t>Deepak Khatri</t>
         </is>
       </c>
       <c r="F48" s="3" t="inlineStr">
@@ -3483,7 +3483,7 @@
       </c>
       <c r="E49" s="5" t="inlineStr">
         <is>
-          <t>Meetraj Solanki, Keval Sanghani, Aditya Patel, Mukesh Goswami, Chandan Kamal, Ganpat Prajapati, Deepak Khatri, Shrey Savaliya, Vidhan Padsala, Keyur Chaniyara, Yatree Ladani</t>
+          <t>Chandan Kamal</t>
         </is>
       </c>
       <c r="F49" s="5" t="inlineStr">
@@ -3545,7 +3545,7 @@
       </c>
       <c r="E50" s="3" t="inlineStr">
         <is>
-          <t>Meetraj Solanki, Keval Sanghani, Aditya Patel, Mukesh Goswami, Chandan Kamal, Ganpat Prajapati, Deepak Khatri, Shrey Savaliya, Vidhan Padsala, Keyur Chaniyara, Yatree Ladani</t>
+          <t>Mukesh Goswami</t>
         </is>
       </c>
       <c r="F50" s="3" t="inlineStr">
@@ -3607,7 +3607,7 @@
       </c>
       <c r="E51" s="5" t="inlineStr">
         <is>
-          <t>Meetraj Solanki, Keval Sanghani, Aditya Patel, Mukesh Goswami, Chandan Kamal, Ganpat Prajapati, Deepak Khatri, Shrey Savaliya, Vidhan Padsala, Keyur Chaniyara, Yatree Ladani</t>
+          <t>Shrey Savaliya</t>
         </is>
       </c>
       <c r="F51" s="5" t="inlineStr">
@@ -3669,7 +3669,7 @@
       </c>
       <c r="E52" s="3" t="inlineStr">
         <is>
-          <t>Meetraj Solanki, Keval Sanghani, Aditya Patel, Mukesh Goswami, Chandan Kamal, Ganpat Prajapati, Deepak Khatri, Shrey Savaliya, Vidhan Padsala, Keyur Chaniyara, Yatree Ladani</t>
+          <t>Yatree Ladani</t>
         </is>
       </c>
       <c r="F52" s="3" t="inlineStr">
@@ -3731,7 +3731,7 @@
       </c>
       <c r="E53" s="5" t="inlineStr">
         <is>
-          <t>Meetraj Solanki, Keval Sanghani, Aditya Patel, Mukesh Goswami, Chandan Kamal, Ganpat Prajapati, Deepak Khatri, Shrey Savaliya, Vidhan Padsala, Keyur Chaniyara, Yatree Ladani</t>
+          <t>Keval Sanghani</t>
         </is>
       </c>
       <c r="F53" s="5" t="inlineStr">
@@ -3793,7 +3793,7 @@
       </c>
       <c r="E54" s="3" t="inlineStr">
         <is>
-          <t>Meetraj Solanki, Keval Sanghani, Aditya Patel, Mukesh Goswami, Chandan Kamal, Ganpat Prajapati, Deepak Khatri, Shrey Savaliya, Vidhan Padsala, Keyur Chaniyara, Yatree Ladani</t>
+          <t>Meetraj Solanki</t>
         </is>
       </c>
       <c r="F54" s="3" t="inlineStr">
@@ -3855,7 +3855,7 @@
       </c>
       <c r="E55" s="5" t="inlineStr">
         <is>
-          <t>Meetraj Solanki, Keval Sanghani, Aditya Patel, Mukesh Goswami, Chandan Kamal, Ganpat Prajapati, Deepak Khatri, Shrey Savaliya, Vidhan Padsala, Keyur Chaniyara, Yatree Ladani</t>
+          <t>Aditya Patel</t>
         </is>
       </c>
       <c r="F55" s="5" t="inlineStr">
@@ -3917,7 +3917,7 @@
       </c>
       <c r="E56" s="3" t="inlineStr">
         <is>
-          <t>Meetraj Solanki, Keval Sanghani, Aditya Patel, Mukesh Goswami, Chandan Kamal, Ganpat Prajapati, Deepak Khatri, Shrey Savaliya, Vidhan Padsala, Keyur Chaniyara, Yatree Ladani</t>
+          <t>Vidhan Padsala</t>
         </is>
       </c>
       <c r="F56" s="3" t="inlineStr">
@@ -3979,7 +3979,7 @@
       </c>
       <c r="E57" s="5" t="inlineStr">
         <is>
-          <t>Meetraj Solanki, Keval Sanghani, Aditya Patel, Mukesh Goswami, Chandan Kamal, Ganpat Prajapati, Deepak Khatri, Shrey Savaliya, Vidhan Padsala, Keyur Chaniyara, Yatree Ladani</t>
+          <t>Keyur Chaniyara</t>
         </is>
       </c>
       <c r="F57" s="5" t="inlineStr">
@@ -4041,7 +4041,7 @@
       </c>
       <c r="E58" s="3" t="inlineStr">
         <is>
-          <t>Meetraj Solanki, Keval Sanghani, Aditya Patel, Mukesh Goswami, Chandan Kamal, Ganpat Prajapati, Deepak Khatri, Shrey Savaliya, Vidhan Padsala, Keyur Chaniyara, Yatree Ladani</t>
+          <t>Ganpat Prajapati</t>
         </is>
       </c>
       <c r="F58" s="3" t="inlineStr">
@@ -4103,7 +4103,7 @@
       </c>
       <c r="E59" s="5" t="inlineStr">
         <is>
-          <t>Meetraj Solanki, Keval Sanghani, Aditya Patel, Mukesh Goswami, Chandan Kamal, Ganpat Prajapati, Deepak Khatri, Shrey Savaliya, Vidhan Padsala, Keyur Chaniyara, Yatree Ladani</t>
+          <t>Deepak Khatri</t>
         </is>
       </c>
       <c r="F59" s="5" t="inlineStr">
@@ -4165,7 +4165,7 @@
       </c>
       <c r="E60" s="3" t="inlineStr">
         <is>
-          <t>Meetraj Solanki, Keval Sanghani, Aditya Patel, Mukesh Goswami, Chandan Kamal, Ganpat Prajapati, Deepak Khatri, Shrey Savaliya, Vidhan Padsala, Keyur Chaniyara, Yatree Ladani</t>
+          <t>Chandan Kamal</t>
         </is>
       </c>
       <c r="F60" s="3" t="inlineStr">
@@ -4227,7 +4227,7 @@
       </c>
       <c r="E61" s="5" t="inlineStr">
         <is>
-          <t>Meetraj Solanki, Keval Sanghani, Aditya Patel, Mukesh Goswami, Chandan Kamal, Ganpat Prajapati, Deepak Khatri, Shrey Savaliya, Vidhan Padsala, Keyur Chaniyara, Yatree Ladani</t>
+          <t>Mukesh Goswami</t>
         </is>
       </c>
       <c r="F61" s="5" t="inlineStr">

</xml_diff>